<commit_message>
"Vorlesung besucht?"-Spalte korrigieren: nur VA-Tage sind "ja"
Bug gefunden vom Nutzer: die Spalte stand bislang auf "ja" für jeden
Tag außer Typ A - also fälschlich auch an allen 6 Feiertagen, beiden
Krankheitstagen und sogar an Wochenend-Zeilen. Weder an Feiertagen noch
im Krankheitsfall wurde eine Vorlesung besucht.

ws.cell(r, 7).value setzt jetzt "ja" nur noch für typ == "VA", "nein"
für A/F/K, und bleibt leer für Wochenendzeilen (wie Spalte Typ/Stunden
dort auch leer sind).

Reine Korrektur einer Anzeige-Spalte, die von keinem anderen Skript
gelesen wird - Stunden, Typen und Zeiterfassung unverändert bei 740,00 h.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U4BNk3uadsQpTDXBqWzPi1
</commit_message>
<xml_diff>
--- a/hochschule/Hassine_3399727_Tätigkeitsnachweis.xlsx
+++ b/hochschule/Hassine_3399727_Tätigkeitsnachweis.xlsx
@@ -3997,11 +3997,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G21" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G21" s="96" t="n"/>
       <c r="H21" s="67" t="n"/>
       <c r="I21" s="86" t="n"/>
       <c r="J21" s="86" t="n"/>
@@ -4029,11 +4025,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G22" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G22" s="96" t="n"/>
       <c r="H22" s="67" t="n"/>
       <c r="I22" s="86" t="n"/>
       <c r="J22" s="86" t="n"/>
@@ -4271,11 +4263,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G28" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G28" s="96" t="n"/>
       <c r="H28" s="67" t="n"/>
       <c r="I28" s="86" t="n"/>
       <c r="J28" s="86" t="n"/>
@@ -4303,11 +4291,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G29" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G29" s="96" t="n"/>
       <c r="H29" s="67" t="n"/>
       <c r="I29" s="86" t="n"/>
       <c r="J29" s="86" t="n"/>
@@ -4509,7 +4493,7 @@
       </c>
       <c r="G34" s="96" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H34" s="67" t="inlineStr">
@@ -4543,11 +4527,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G35" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G35" s="96" t="n"/>
       <c r="H35" s="67" t="n"/>
       <c r="I35" s="86" t="n"/>
       <c r="J35" s="86" t="n"/>
@@ -4575,11 +4555,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G36" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G36" s="96" t="n"/>
       <c r="H36" s="67" t="n"/>
       <c r="I36" s="86" t="n"/>
       <c r="J36" s="86" t="n"/>
@@ -4812,11 +4788,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G42" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G42" s="96" t="n"/>
       <c r="H42" s="67" t="n"/>
       <c r="I42" s="86" t="n"/>
       <c r="J42" s="86" t="n"/>
@@ -4843,11 +4815,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G43" s="13" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G43" s="13" t="n"/>
       <c r="H43" s="74" t="n"/>
       <c r="I43" s="86" t="n"/>
       <c r="J43" s="86" t="n"/>
@@ -5358,7 +5326,7 @@
       </c>
       <c r="G63" s="96" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H63" s="67" t="inlineStr">
@@ -5391,11 +5359,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G64" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G64" s="96" t="n"/>
       <c r="H64" s="67" t="n"/>
       <c r="I64" s="86" t="n"/>
       <c r="J64" s="86" t="n"/>
@@ -5422,11 +5386,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G65" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G65" s="96" t="n"/>
       <c r="H65" s="67" t="n"/>
       <c r="I65" s="86" t="n"/>
       <c r="J65" s="86" t="n"/>
@@ -5459,7 +5419,7 @@
       </c>
       <c r="G66" s="96" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H66" s="94" t="inlineStr">
@@ -5656,11 +5616,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G71" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G71" s="96" t="n"/>
       <c r="H71" s="67" t="n"/>
       <c r="I71" s="86" t="n"/>
       <c r="J71" s="86" t="n"/>
@@ -5687,11 +5643,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G72" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G72" s="96" t="n"/>
       <c r="H72" s="67" t="n"/>
       <c r="I72" s="86" t="n"/>
       <c r="J72" s="86" t="n"/>
@@ -5923,11 +5875,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G78" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G78" s="96" t="n"/>
       <c r="H78" s="67" t="n"/>
       <c r="I78" s="86" t="n"/>
       <c r="J78" s="86" t="n"/>
@@ -5954,11 +5902,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G79" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G79" s="96" t="n"/>
       <c r="H79" s="67" t="n"/>
       <c r="I79" s="86" t="n"/>
       <c r="J79" s="86" t="n"/>
@@ -6190,11 +6134,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G85" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G85" s="96" t="n"/>
       <c r="H85" s="67" t="n"/>
       <c r="I85" s="86" t="n"/>
       <c r="J85" s="86" t="n"/>
@@ -6221,11 +6161,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G86" s="13" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G86" s="13" t="n"/>
       <c r="H86" s="74" t="n"/>
       <c r="I86" s="86" t="n"/>
       <c r="J86" s="86" t="n"/>
@@ -6736,7 +6672,7 @@
       </c>
       <c r="G106" s="96" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H106" s="67" t="inlineStr">
@@ -6769,11 +6705,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G107" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G107" s="96" t="n"/>
       <c r="H107" s="67" t="n"/>
       <c r="I107" s="86" t="n"/>
       <c r="J107" s="86" t="n"/>
@@ -6800,11 +6732,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G108" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G108" s="96" t="n"/>
       <c r="H108" s="67" t="n"/>
       <c r="I108" s="86" t="n"/>
       <c r="J108" s="86" t="n"/>
@@ -7036,11 +6964,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G114" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G114" s="96" t="n"/>
       <c r="H114" s="67" t="n"/>
       <c r="I114" s="86" t="n"/>
       <c r="J114" s="86" t="n"/>
@@ -7067,11 +6991,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G115" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G115" s="96" t="n"/>
       <c r="H115" s="67" t="n"/>
       <c r="I115" s="86" t="n"/>
       <c r="J115" s="86" t="n"/>
@@ -7227,7 +7147,7 @@
       </c>
       <c r="G119" s="96" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H119" s="94" t="inlineStr">
@@ -7301,11 +7221,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G121" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G121" s="96" t="n"/>
       <c r="H121" s="67" t="n"/>
       <c r="I121" s="86" t="n"/>
       <c r="J121" s="86" t="n"/>
@@ -7332,11 +7248,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G122" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G122" s="96" t="n"/>
       <c r="H122" s="67" t="n"/>
       <c r="I122" s="86" t="n"/>
       <c r="J122" s="86" t="n"/>
@@ -7568,11 +7480,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G128" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G128" s="96" t="n"/>
       <c r="H128" s="67" t="n"/>
       <c r="I128" s="86" t="n"/>
       <c r="J128" s="86" t="n"/>
@@ -7599,11 +7507,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G129" s="13" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G129" s="13" t="n"/>
       <c r="H129" s="74" t="n"/>
       <c r="I129" s="86" t="n"/>
       <c r="J129" s="86" t="n"/>
@@ -7950,7 +7854,7 @@
       </c>
       <c r="G145" s="8" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H145" s="94" t="inlineStr">
@@ -8147,11 +8051,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G150" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G150" s="96" t="n"/>
       <c r="H150" s="67" t="n"/>
       <c r="I150" s="86" t="n"/>
       <c r="J150" s="86" t="n"/>
@@ -8178,11 +8078,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G151" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G151" s="96" t="n"/>
       <c r="H151" s="67" t="n"/>
       <c r="I151" s="86" t="n"/>
       <c r="J151" s="86" t="n"/>
@@ -8338,7 +8234,7 @@
       </c>
       <c r="G155" s="96" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H155" s="94" t="inlineStr">
@@ -8412,11 +8308,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G157" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G157" s="96" t="n"/>
       <c r="H157" s="67" t="n"/>
       <c r="I157" s="86" t="n"/>
       <c r="J157" s="86" t="n"/>
@@ -8443,11 +8335,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G158" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G158" s="96" t="n"/>
       <c r="H158" s="67" t="n"/>
       <c r="I158" s="86" t="n"/>
       <c r="J158" s="86" t="n"/>
@@ -8679,11 +8567,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G164" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G164" s="96" t="n"/>
       <c r="H164" s="67" t="n"/>
       <c r="I164" s="86" t="n"/>
       <c r="J164" s="86" t="n"/>
@@ -8710,11 +8594,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G165" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G165" s="96" t="n"/>
       <c r="H165" s="67" t="n"/>
       <c r="I165" s="86" t="n"/>
       <c r="J165" s="86" t="n"/>
@@ -8946,11 +8826,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G171" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G171" s="96" t="n"/>
       <c r="H171" s="67" t="n"/>
       <c r="I171" s="86" t="n"/>
       <c r="J171" s="86" t="n"/>
@@ -8977,11 +8853,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G172" s="13" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G172" s="13" t="n"/>
       <c r="H172" s="74" t="n"/>
       <c r="I172" s="86" t="n"/>
       <c r="J172" s="86" t="n"/>
@@ -9527,11 +9399,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G193" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G193" s="96" t="n"/>
       <c r="H193" s="67" t="n"/>
       <c r="I193" s="86" t="n"/>
       <c r="J193" s="86" t="n"/>
@@ -9558,11 +9426,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G194" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G194" s="96" t="n"/>
       <c r="H194" s="67" t="n"/>
       <c r="I194" s="86" t="n"/>
       <c r="J194" s="86" t="n"/>
@@ -9759,7 +9623,7 @@
       </c>
       <c r="G199" s="96" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>nein</t>
         </is>
       </c>
       <c r="H199" s="98" t="inlineStr">
@@ -9792,11 +9656,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G200" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G200" s="96" t="n"/>
       <c r="H200" s="67" t="n"/>
       <c r="I200" s="86" t="n"/>
       <c r="J200" s="86" t="n"/>
@@ -9823,11 +9683,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G201" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G201" s="96" t="n"/>
       <c r="H201" s="67" t="n"/>
       <c r="I201" s="86" t="n"/>
       <c r="J201" s="86" t="n"/>
@@ -10059,11 +9915,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G207" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G207" s="96" t="n"/>
       <c r="H207" s="67" t="n"/>
       <c r="I207" s="86" t="n"/>
       <c r="J207" s="86" t="n"/>
@@ -10090,11 +9942,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G208" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G208" s="96" t="n"/>
       <c r="H208" s="67" t="n"/>
       <c r="I208" s="86" t="n"/>
       <c r="J208" s="86" t="n"/>
@@ -10326,11 +10174,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G214" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G214" s="96" t="n"/>
       <c r="H214" s="67" t="n"/>
       <c r="I214" s="86" t="n"/>
       <c r="J214" s="86" t="n"/>
@@ -10357,11 +10201,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G215" s="13" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G215" s="13" t="n"/>
       <c r="H215" s="74" t="n"/>
       <c r="I215" s="86" t="n"/>
       <c r="J215" s="86" t="n"/>
@@ -10907,11 +10747,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G236" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G236" s="96" t="n"/>
       <c r="H236" s="67" t="n"/>
       <c r="I236" s="86" t="n"/>
       <c r="J236" s="86" t="n"/>
@@ -10938,11 +10774,7 @@
           <t>h</t>
         </is>
       </c>
-      <c r="G237" s="96" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
+      <c r="G237" s="96" t="n"/>
       <c r="H237" s="67" t="n"/>
       <c r="I237" s="86" t="n"/>
       <c r="J237" s="86" t="n"/>

</xml_diff>